<commit_message>
Sync from vault 2026-06-01 17:52:50
</commit_message>
<xml_diff>
--- a/content/Radio/Atmos Klassiek/0. Files/Playlist weights.xlsx
+++ b/content/Radio/Atmos Klassiek/0. Files/Playlist weights.xlsx
@@ -82,40 +82,40 @@
     <t xml:space="preserve">jingles-pre-ad</t>
   </si>
   <si>
+    <t xml:space="preserve">Klassiek-fanfare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nacht-klassiek-inspired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
     <t xml:space="preserve">klassiek-ghibli</t>
   </si>
   <si>
-    <t xml:space="preserve">nacht-klassiek-inspired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
+    <t xml:space="preserve">nacht-luit</t>
   </si>
   <si>
     <t xml:space="preserve">klassiek-hits</t>
   </si>
   <si>
-    <t xml:space="preserve">nacht-luit</t>
+    <t xml:space="preserve">nacht-regency</t>
   </si>
   <si>
     <t xml:space="preserve">klassiek-inspired</t>
   </si>
   <si>
-    <t xml:space="preserve">nacht-regency</t>
+    <t xml:space="preserve">nacht-tango</t>
   </si>
   <si>
     <t xml:space="preserve">klassiek-luit</t>
   </si>
   <si>
-    <t xml:space="preserve">nacht-tango</t>
-  </si>
-  <si>
     <t xml:space="preserve">klassiek-regency</t>
   </si>
   <si>
     <t xml:space="preserve">klassiek-tango</t>
-  </si>
-  <si>
-    <t xml:space="preserve">klassiek-zang</t>
   </si>
 </sst>
 </file>
@@ -248,8 +248,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="daytime" displayName="daytime" ref="A1:E12" headerRowCount="1" totalsRowCount="1" totalsRowShown="1">
-  <autoFilter ref="A1:E12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="daytime" displayName="daytime" ref="A1:E11" headerRowCount="1" totalsRowCount="1" totalsRowShown="1">
+  <autoFilter ref="A1:E11"/>
   <tableColumns count="5">
     <tableColumn id="1" name="List"/>
     <tableColumn id="2" name="Weight"/>
@@ -291,7 +291,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:X1048576"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.42"/>
@@ -306,16 +306,16 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="8.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="7.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="7.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="10.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="15.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="15.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="9.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="0" width="7.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="0" width="7.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="25" style="0" width="8.48"/>
   </cols>
   <sheetData>
@@ -384,7 +384,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>8</v>
       </c>
@@ -395,29 +395,29 @@
         <v>19</v>
       </c>
       <c r="D2" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.1</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.121212121212121</v>
       </c>
       <c r="E2" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00526315789473684</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00637958532695375</v>
       </c>
       <c r="G2" s="0" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="0" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2" s="0" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.0731707317073171</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.0357142857142857</v>
       </c>
       <c r="K2" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.0182926829268293</v>
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.0357142857142857</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>10</v>
@@ -426,7 +426,7 @@
         <v>5</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P2" s="4" t="n">
         <f aca="false">ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]]</f>
@@ -434,11 +434,11 @@
       </c>
       <c r="Q2" s="4" t="n">
         <f aca="false">(ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]])/ads[[#This Row],[Length]]</f>
-        <v>0.0714285714285714</v>
+        <v>0.0555555555555556</v>
       </c>
       <c r="R2" s="4" t="n">
         <f aca="false">ads[[#This Row],[%/ad]]*4</f>
-        <v>0.285714285714286</v>
+        <v>0.222222222222222</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>11</v>
@@ -458,7 +458,7 @@
         <v>0.166666666666667</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>12</v>
       </c>
@@ -469,29 +469,29 @@
         <v>33</v>
       </c>
       <c r="D3" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.05</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0606060606060606</v>
       </c>
       <c r="E3" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00151515151515152</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00183654729109275</v>
       </c>
       <c r="G3" s="0" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="0" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I3" s="0" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J3" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.24390243902439</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.214285714285714</v>
       </c>
       <c r="K3" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.024390243902439</v>
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.00857142857142857</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>14</v>
@@ -500,7 +500,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P3" s="4" t="n">
         <f aca="false">ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]]</f>
@@ -508,11 +508,11 @@
       </c>
       <c r="Q3" s="4" t="n">
         <f aca="false">(ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]])/ads[[#This Row],[Length]]</f>
-        <v>0.0125</v>
+        <v>0.01</v>
       </c>
       <c r="R3" s="4" t="n">
         <f aca="false">ads[[#This Row],[%/ad]]*4</f>
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="T3" s="3" t="s">
         <v>15</v>
@@ -532,40 +532,40 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.05</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0909090909090909</v>
       </c>
       <c r="E4" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00625</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00505050505050505</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>17</v>
       </c>
       <c r="H4" s="0" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I4" s="0" t="n">
         <v>21</v>
       </c>
       <c r="J4" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.170731707317073</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.178571428571429</v>
       </c>
       <c r="K4" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.00813008130081301</v>
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.00850340136054422</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>18</v>
@@ -574,7 +574,7 @@
         <v>4</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P4" s="4" t="n">
         <f aca="false">ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]]</f>
@@ -582,11 +582,11 @@
       </c>
       <c r="Q4" s="4" t="n">
         <f aca="false">(ads[[#This Row],[Weight]]/ads[[#Totals],[Weight]])/ads[[#This Row],[Length]]</f>
-        <v>0.04</v>
+        <v>0.0444444444444444</v>
       </c>
       <c r="R4" s="4" t="n">
         <f aca="false">ads[[#This Row],[%/ad]]*4</f>
-        <v>0.16</v>
+        <v>0.177777777777778</v>
       </c>
       <c r="T4" s="3" t="s">
         <v>19</v>
@@ -606,40 +606,40 @@
         <v>0.0833333333333333</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="0" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.1</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0909090909090909</v>
       </c>
       <c r="E5" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00294117647058823</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.0025974025974026</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>21</v>
       </c>
       <c r="H5" s="0" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I5" s="0" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="J5" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.219512195121951</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.25</v>
       </c>
       <c r="K5" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.00878048780487805</v>
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.00862068965517241</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>22</v>
@@ -650,7 +650,7 @@
       </c>
       <c r="O5" s="3" t="n">
         <f aca="false">SUBTOTAL(109,ads[Length])</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
@@ -669,43 +669,43 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="0" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C6" s="0" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="D6" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.25</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.121212121212121</v>
       </c>
       <c r="E6" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.015625</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.0035650623885918</v>
       </c>
       <c r="G6" s="0" t="s">
         <v>24</v>
       </c>
       <c r="H6" s="0" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>26</v>
       </c>
       <c r="J6" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.195121951219512</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.178571428571429</v>
       </c>
       <c r="K6" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.0075046904315197</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.00686813186813187</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
         <v>25</v>
       </c>
@@ -713,15 +713,15 @@
         <v>6</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.15</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.181818181818182</v>
       </c>
       <c r="E7" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00714285714285714</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00673400673400673</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>26</v>
@@ -733,31 +733,31 @@
         <v>8</v>
       </c>
       <c r="J7" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.0731707317073171</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.107142857142857</v>
       </c>
       <c r="K7" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.00914634146341463</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.0133928571428571</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="0" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C8" s="0" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.075</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.181818181818182</v>
       </c>
       <c r="E8" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00267857142857143</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00865800865800866</v>
       </c>
       <c r="G8" s="0" t="s">
         <v>28</v>
@@ -769,100 +769,99 @@
         <v>3</v>
       </c>
       <c r="J8" s="2" t="n">
-        <f aca="false">nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]]</f>
-        <v>0.024390243902439</v>
+        <f aca="false">nighttime[[#This Row],[Weight]]/$H$9</f>
+        <v>0.0357142857142857</v>
       </c>
       <c r="K8" s="2" t="n">
-        <f aca="false">(nighttime[[#This Row],[Weight]]/nighttime[[#Totals],[Weight]])/nighttime[[#This Row],[Length]]</f>
-        <v>0.00813008130081301</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(nighttime[[#This Row],[Weight]]/$H$9)/nighttime[[#This Row],[Length]]</f>
+        <v>0.0119047619047619</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="0" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="0" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D9" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.05</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0909090909090909</v>
       </c>
       <c r="E9" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00357142857142857</v>
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.0034965034965035</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>22</v>
       </c>
       <c r="H9" s="0" t="n">
         <f aca="false">SUBTOTAL(109,nighttime[Weight])</f>
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="I9" s="0" t="n">
         <f aca="false">SUBTOTAL(109,nighttime[Length])</f>
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D10" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.075</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0606060606060606</v>
       </c>
       <c r="E10" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00288461538461538</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.00432900432900433</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
         <v>31</v>
       </c>
       <c r="B11" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D11" s="2" t="n">
-        <f aca="false">daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]]</f>
-        <v>0.1</v>
+        <f aca="false">daytime[[#This Row],[Weight]]/$B$12</f>
+        <v>0.0909090909090909</v>
       </c>
       <c r="E11" s="2" t="n">
-        <f aca="false">(daytime[[#This Row],[Weight]]/daytime[[#Totals],[Weight]])/daytime[[#This Row],[Length]]</f>
-        <v>0.00909090909090909</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(daytime[[#This Row],[Weight]]/$B$12)/daytime[[#This Row],[Length]]</f>
+        <v>0.0034965034965035</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">SUM(daytime[Weight])</f>
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">SUBTOTAL(109,daytime[Length])</f>
-        <v>210</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E13" s="2"/>
-    </row>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <conditionalFormatting sqref="B2:B11">
+  <conditionalFormatting sqref="B2:B5">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -954,6 +953,36 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="X2:X4">
     <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:B12">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D12">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E12">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min" val="0"/>
         <cfvo type="max" val="0"/>

</xml_diff>